<commit_message>
update figures and data
</commit_message>
<xml_diff>
--- a/inst/extdata/wb_projects_gov_afe.xlsx
+++ b/inst/extdata/wb_projects_gov_afe.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="153">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="157">
   <si>
     <t xml:space="preserve">proj_id</t>
   </si>
@@ -52,6 +52,18 @@
   </si>
   <si>
     <t xml:space="preserve">commitment_amount</t>
+  </si>
+  <si>
+    <t xml:space="preserve">theme_pfm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">theme_procurement</t>
+  </si>
+  <si>
+    <t xml:space="preserve">theme_public_admin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">theme_env_social</t>
   </si>
   <si>
     <t xml:space="preserve">comments</t>
@@ -821,7 +833,11 @@
     <col min="11" max="11" width="32.71" hidden="0" customWidth="1"/>
     <col min="12" max="12" width="14.71" hidden="0" customWidth="1"/>
     <col min="13" max="13" width="17.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="8.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="9.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="17.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="18.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="16.71" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="8.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -867,655 +883,847 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>2020</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>19</v>
+        <v>23</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="L2" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="M2" s="1" t="n">
         <v>135000000</v>
       </c>
-      <c r="N2" s="1" t="s">
-        <v>25</v>
+      <c r="N2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>2022</v>
       </c>
       <c r="G3" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I3" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J3" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="L3" s="1" t="s">
         <v>28</v>
-      </c>
-      <c r="H3" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="J3" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="K3" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="L3" s="1" t="s">
-        <v>24</v>
       </c>
       <c r="M3" s="1" t="n">
         <v>62000000</v>
       </c>
-      <c r="N3" s="1" t="s">
-        <v>25</v>
+      <c r="N3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>2024</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>23</v>
+        <v>27</v>
       </c>
       <c r="L4" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="M4" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N4" s="1" t="s">
-        <v>25</v>
+      <c r="N4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R4" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="F5" s="1" t="n">
         <v>2024</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="L5" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="M5" s="1" t="n">
         <v>20000000</v>
       </c>
-      <c r="N5" s="1" t="s">
-        <v>25</v>
+      <c r="N5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R5" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>2024</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I6" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J6" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>44</v>
+        <v>48</v>
       </c>
       <c r="L6" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="M6" s="1" t="n">
         <v>150000000</v>
       </c>
-      <c r="N6" s="1" t="s">
-        <v>25</v>
+      <c r="N6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q6" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R6" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B7" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E7" s="1" t="s">
         <v>45</v>
-      </c>
-      <c r="B7" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>41</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>2024</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="L7" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="M7" s="1" t="n">
         <v>200000000</v>
       </c>
-      <c r="N7" s="1" t="s">
-        <v>25</v>
+      <c r="N7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R7" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>2020</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="L8" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="M8" s="1" t="n">
         <v>100000000</v>
       </c>
-      <c r="N8" s="1" t="s">
-        <v>25</v>
+      <c r="N8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q8" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R8" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="B9" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>56</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="D9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E9" s="1" t="s">
         <v>57</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>53</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>2024</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="L9" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="M9" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N9" s="1" t="s">
-        <v>25</v>
+      <c r="N9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R9" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>61</v>
+        <v>65</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>2026</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>63</v>
+        <v>67</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J10" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="L10" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="M10" s="1"/>
-      <c r="N10" s="1" t="s">
-        <v>25</v>
+      <c r="N10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="P10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R10" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>65</v>
+        <v>69</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>66</v>
+        <v>70</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F11" s="1" t="n">
         <v>2022</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>69</v>
+        <v>73</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J11" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="L11" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="M11" s="1" t="n">
         <v>34000000</v>
       </c>
-      <c r="N11" s="1" t="s">
-        <v>25</v>
+      <c r="N11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="P11" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>71</v>
+        <v>75</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="D12" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E12" s="1" t="s">
         <v>72</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>73</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E12" s="1" t="s">
-        <v>68</v>
       </c>
       <c r="F12" s="1" t="n">
         <v>2025</v>
       </c>
       <c r="G12" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I12" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J12" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="K12" s="1" t="s">
         <v>74</v>
       </c>
-      <c r="H12" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="I12" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="J12" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="K12" s="1" t="s">
-        <v>70</v>
-      </c>
       <c r="L12" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="M12" s="1"/>
-      <c r="N12" s="1" t="s">
-        <v>25</v>
+      <c r="N12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R12" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>75</v>
+        <v>79</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>77</v>
+        <v>81</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F13" s="1" t="n">
         <v>2026</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>79</v>
+        <v>83</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="L13" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="M13" s="1"/>
-      <c r="N13" s="1" t="s">
-        <v>25</v>
+      <c r="N13" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="P13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R13" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>81</v>
+        <v>85</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>82</v>
+        <v>86</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>83</v>
+        <v>87</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F14" s="1" t="n">
         <v>2022</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>85</v>
+        <v>89</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="L14" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="M14" s="1" t="n">
         <v>210000000</v>
       </c>
-      <c r="N14" s="1" t="s">
-        <v>25</v>
+      <c r="N14" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R14" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>87</v>
+        <v>91</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>88</v>
+        <v>92</v>
       </c>
       <c r="C15" s="1"/>
       <c r="D15" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="F15" s="1" t="n">
         <v>2024</v>
       </c>
       <c r="G15" s="1" t="s">
-        <v>90</v>
+        <v>94</v>
       </c>
       <c r="H15" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K15" s="1" t="s">
-        <v>91</v>
+        <v>95</v>
       </c>
       <c r="L15" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="M15" s="1" t="n">
         <v>0</v>
       </c>
-      <c r="N15" s="1" t="s">
-        <v>25</v>
+      <c r="N15" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O15" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P15" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q15" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R15" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="B16" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="D16" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E16" s="1" t="s">
         <v>93</v>
-      </c>
-      <c r="C16" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="D16" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E16" s="1" t="s">
-        <v>89</v>
       </c>
       <c r="F16" s="1" t="n">
         <v>2024</v>
       </c>
       <c r="G16" s="1" t="s">
-        <v>95</v>
+        <v>99</v>
       </c>
       <c r="H16" s="1" t="s">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>21</v>
+        <v>25</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K16" s="1" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="L16" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="M16" s="1"/>
-      <c r="N16" s="1" t="s">
-        <v>25</v>
+      <c r="N16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P16" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q16" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R16" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>
@@ -1542,7 +1750,11 @@
     <col min="11" max="11" width="35.71" hidden="0" customWidth="1"/>
     <col min="12" max="12" width="14.71" hidden="0" customWidth="1"/>
     <col min="13" max="13" width="17.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="8.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="9.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="17.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="18.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="16.71" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="8.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1588,489 +1800,657 @@
       <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
+      <c r="O1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>97</v>
+        <v>101</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>98</v>
+        <v>102</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>99</v>
+        <v>103</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>100</v>
+        <v>104</v>
       </c>
       <c r="F2" s="1" t="n">
         <v>2027</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>101</v>
+        <v>105</v>
       </c>
       <c r="H2" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I2" s="1"/>
       <c r="J2" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="L2" s="1"/>
       <c r="M2" s="1"/>
-      <c r="N2" s="1" t="s">
-        <v>25</v>
+      <c r="N2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q2" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R2" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="B3" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E3" s="1" t="s">
         <v>104</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>105</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>106</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>100</v>
       </c>
       <c r="F3" s="1" t="n">
         <v>2027</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>107</v>
+        <v>111</v>
       </c>
       <c r="H3" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I3" s="1"/>
       <c r="J3" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>103</v>
+        <v>107</v>
       </c>
       <c r="L3" s="1"/>
       <c r="M3" s="1"/>
-      <c r="N3" s="1" t="s">
-        <v>25</v>
+      <c r="N3" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>108</v>
+        <v>112</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>109</v>
+        <v>113</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>110</v>
+        <v>114</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F4" s="1" t="n">
         <v>2028</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="H4" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I4" s="1"/>
       <c r="J4" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K4" s="1" t="s">
-        <v>112</v>
+        <v>116</v>
       </c>
       <c r="L4" s="1"/>
       <c r="M4" s="1"/>
-      <c r="N4" s="1" t="s">
-        <v>25</v>
+      <c r="N4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q4" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R4" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>113</v>
+        <v>117</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>114</v>
+        <v>118</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>115</v>
+        <v>119</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="F5" s="1" t="n">
         <v>2028</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="H5" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I5" s="1"/>
       <c r="J5" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K5" s="1" t="s">
-        <v>80</v>
+        <v>84</v>
       </c>
       <c r="L5" s="1"/>
       <c r="M5" s="1"/>
-      <c r="N5" s="1" t="s">
-        <v>25</v>
+      <c r="N5" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q5" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R5" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1" t="s">
-        <v>117</v>
+        <v>121</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>118</v>
+        <v>122</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>119</v>
+        <v>123</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>120</v>
+        <v>124</v>
       </c>
       <c r="F6" s="1" t="n">
         <v>2018</v>
       </c>
       <c r="G6" s="1" t="s">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="H6" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I6" s="1"/>
       <c r="J6" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>122</v>
+        <v>126</v>
       </c>
       <c r="L6" s="1"/>
       <c r="M6" s="1"/>
-      <c r="N6" s="1" t="s">
-        <v>25</v>
+      <c r="N6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q6" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R6" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>123</v>
+        <v>127</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>125</v>
+        <v>129</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F7" s="1" t="n">
         <v>2027</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>126</v>
+        <v>130</v>
       </c>
       <c r="H7" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I7" s="1"/>
       <c r="J7" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K7" s="1" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="L7" s="1"/>
       <c r="M7" s="1"/>
-      <c r="N7" s="1" t="s">
-        <v>25</v>
+      <c r="N7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q7" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="R7" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="s">
-        <v>127</v>
+        <v>131</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>128</v>
+        <v>132</v>
       </c>
       <c r="C8" s="1"/>
       <c r="D8" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="F8" s="1" t="n">
         <v>2026</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>129</v>
+        <v>133</v>
       </c>
       <c r="H8" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I8" s="1"/>
       <c r="J8" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K8" s="1" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="L8" s="1"/>
       <c r="M8" s="1"/>
-      <c r="N8" s="1" t="s">
-        <v>25</v>
+      <c r="N8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q8" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R8" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1" t="s">
-        <v>130</v>
+        <v>134</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>131</v>
+        <v>135</v>
       </c>
       <c r="C9" s="1"/>
       <c r="D9" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>62</v>
+        <v>66</v>
       </c>
       <c r="F9" s="1" t="n">
         <v>2027</v>
       </c>
       <c r="G9" s="1" t="s">
-        <v>132</v>
+        <v>136</v>
       </c>
       <c r="H9" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I9" s="1"/>
       <c r="J9" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K9" s="1" t="s">
-        <v>64</v>
+        <v>68</v>
       </c>
       <c r="L9" s="1"/>
       <c r="M9" s="1"/>
-      <c r="N9" s="1" t="s">
-        <v>25</v>
+      <c r="N9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P9" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q9" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R9" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>133</v>
+        <v>137</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>134</v>
+        <v>138</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>135</v>
+        <v>139</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>68</v>
+        <v>72</v>
       </c>
       <c r="F10" s="1" t="n">
         <v>2027</v>
       </c>
       <c r="G10" s="1" t="s">
-        <v>136</v>
+        <v>140</v>
       </c>
       <c r="H10" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I10" s="1"/>
       <c r="J10" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="L10" s="1"/>
       <c r="M10" s="1"/>
-      <c r="N10" s="1" t="s">
-        <v>25</v>
+      <c r="N10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P10" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="Q10" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R10" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>137</v>
+        <v>141</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="C11" s="1"/>
       <c r="D11" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>78</v>
+        <v>82</v>
       </c>
       <c r="F11" s="1" t="n">
         <v>2026</v>
       </c>
       <c r="G11" s="1" t="s">
-        <v>139</v>
+        <v>143</v>
       </c>
       <c r="H11" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I11" s="1"/>
       <c r="J11" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>140</v>
+        <v>144</v>
       </c>
       <c r="L11" s="1"/>
       <c r="M11" s="1"/>
-      <c r="N11" s="1" t="s">
-        <v>25</v>
+      <c r="N11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q11" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R11" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1" t="s">
-        <v>141</v>
+        <v>145</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>142</v>
+        <v>146</v>
       </c>
       <c r="C12" s="1"/>
       <c r="D12" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F12" s="1" t="n">
         <v>2026</v>
       </c>
       <c r="G12" s="1" t="s">
-        <v>143</v>
+        <v>147</v>
       </c>
       <c r="H12" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I12" s="1"/>
       <c r="J12" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K12" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="L12" s="1"/>
       <c r="M12" s="1"/>
-      <c r="N12" s="1" t="s">
-        <v>25</v>
+      <c r="N12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q12" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R12" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>144</v>
+        <v>148</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>145</v>
+        <v>149</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>146</v>
+        <v>150</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>147</v>
+        <v>151</v>
       </c>
       <c r="F13" s="1" t="n">
         <v>2027</v>
       </c>
       <c r="G13" s="1" t="s">
-        <v>148</v>
+        <v>152</v>
       </c>
       <c r="H13" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I13" s="1"/>
       <c r="J13" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K13" s="1" t="s">
-        <v>149</v>
+        <v>153</v>
       </c>
       <c r="L13" s="1"/>
       <c r="M13" s="1"/>
-      <c r="N13" s="1" t="s">
-        <v>25</v>
+      <c r="N13" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q13" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R13" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>150</v>
+        <v>154</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>151</v>
+        <v>155</v>
       </c>
       <c r="C14" s="1"/>
       <c r="D14" s="1" t="s">
-        <v>17</v>
+        <v>21</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>89</v>
+        <v>93</v>
       </c>
       <c r="F14" s="1" t="n">
         <v>2026</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="H14" s="1" t="s">
-        <v>102</v>
+        <v>106</v>
       </c>
       <c r="I14" s="1"/>
       <c r="J14" s="1" t="s">
-        <v>22</v>
+        <v>26</v>
       </c>
       <c r="K14" s="1" t="s">
-        <v>86</v>
+        <v>90</v>
       </c>
       <c r="L14" s="1"/>
       <c r="M14" s="1"/>
-      <c r="N14" s="1" t="s">
-        <v>25</v>
+      <c r="N14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="P14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="1" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="1" t="s">
+        <v>29</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
exclude 2 ASAs missing approval FY
</commit_message>
<xml_diff>
--- a/inst/extdata/wb_projects_gov_afe.xlsx
+++ b/inst/extdata/wb_projects_gov_afe.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="161" uniqueCount="161">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="164">
   <si>
     <t xml:space="preserve">proj_id</t>
   </si>
@@ -72,6 +72,9 @@
     <t xml:space="preserve">theme_env_social</t>
   </si>
   <si>
+    <t xml:space="preserve">ida_cycle_approval</t>
+  </si>
+  <si>
     <t xml:space="preserve">comments</t>
   </si>
   <si>
@@ -108,6 +111,9 @@
     <t xml:space="preserve">IDA</t>
   </si>
   <si>
+    <t xml:space="preserve">Pre-IDA21</t>
+  </si>
+  <si>
     <t xml:space="preserve"/>
   </si>
   <si>
@@ -226,6 +232,9 @@
   </si>
   <si>
     <t xml:space="preserve">Meron Tadesse Techane (ADM)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IDA21</t>
   </si>
   <si>
     <t xml:space="preserve">P176761</t>
@@ -854,7 +863,8 @@
     <col min="17" max="17" width="17.71" hidden="0" customWidth="1"/>
     <col min="18" max="18" width="18.71" hidden="0" customWidth="1"/>
     <col min="19" max="19" width="16.71" hidden="0" customWidth="1"/>
-    <col min="20" max="20" width="8.71" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="18.71" hidden="0" customWidth="1"/>
+    <col min="21" max="21" width="8.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -918,22 +928,25 @@
       <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="U1" s="2" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>2020</v>
@@ -941,22 +954,22 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O2" s="2" t="n">
         <v>135000000</v>
@@ -974,24 +987,27 @@
         <v>0</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>2022</v>
@@ -999,22 +1015,22 @@
       <c r="G3" s="2"/>
       <c r="H3" s="2"/>
       <c r="I3" s="2" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K3" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L3" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N3" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O3" s="2" t="n">
         <v>62000000</v>
@@ -1032,24 +1048,27 @@
         <v>1</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>2024</v>
@@ -1057,22 +1076,22 @@
       <c r="G4" s="2"/>
       <c r="H4" s="2"/>
       <c r="I4" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O4" s="2" t="n">
         <v>0</v>
@@ -1090,24 +1109,27 @@
         <v>1</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U4" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>2024</v>
@@ -1115,22 +1137,22 @@
       <c r="G5" s="2"/>
       <c r="H5" s="2"/>
       <c r="I5" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O5" s="2" t="n">
         <v>20000000</v>
@@ -1148,24 +1170,27 @@
         <v>1</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U5" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>2024</v>
@@ -1173,22 +1198,22 @@
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O6" s="2" t="n">
         <v>150000000</v>
@@ -1206,24 +1231,27 @@
         <v>1</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U6" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>2024</v>
@@ -1231,22 +1259,22 @@
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
       <c r="I7" s="2" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K7" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="L7" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O7" s="2" t="n">
         <v>200000000</v>
@@ -1264,24 +1292,27 @@
         <v>1</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U7" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>2020</v>
@@ -1289,22 +1320,22 @@
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O8" s="2" t="n">
         <v>100000000</v>
@@ -1322,24 +1353,27 @@
         <v>1</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U8" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>2024</v>
@@ -1347,22 +1381,22 @@
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
       <c r="I9" s="2" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O9" s="2" t="n">
         <v>0</v>
@@ -1380,24 +1414,27 @@
         <v>1</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U9" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>2026</v>
@@ -1405,22 +1442,22 @@
       <c r="G10" s="2"/>
       <c r="H10" s="2"/>
       <c r="I10" s="2" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O10" s="2"/>
       <c r="P10" s="2" t="n">
@@ -1436,24 +1473,27 @@
         <v>1</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>31</v>
+        <v>73</v>
+      </c>
+      <c r="U10" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>73</v>
+        <v>76</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F11" s="2" t="n">
         <v>2022</v>
@@ -1461,22 +1501,22 @@
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2" t="s">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O11" s="2" t="n">
         <v>34000000</v>
@@ -1494,24 +1534,27 @@
         <v>0</v>
       </c>
       <c r="T11" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U11" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
+        <v>80</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>81</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>82</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E12" s="2" t="s">
         <v>77</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>78</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>74</v>
       </c>
       <c r="F12" s="2" t="n">
         <v>2025</v>
@@ -1519,22 +1562,22 @@
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O12" s="2"/>
       <c r="P12" s="2" t="n">
@@ -1550,24 +1593,27 @@
         <v>1</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U12" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>81</v>
+        <v>84</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>2026</v>
@@ -1575,22 +1621,22 @@
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
       <c r="I13" s="2" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O13" s="2"/>
       <c r="P13" s="2" t="n">
@@ -1606,24 +1652,27 @@
         <v>1</v>
       </c>
       <c r="T13" s="2" t="s">
-        <v>31</v>
+        <v>73</v>
+      </c>
+      <c r="U13" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>87</v>
+        <v>90</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>2022</v>
@@ -1631,22 +1680,22 @@
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O14" s="2" t="n">
         <v>210000000</v>
@@ -1664,22 +1713,25 @@
         <v>1</v>
       </c>
       <c r="T14" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U14" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="F15" s="2" t="n">
         <v>2024</v>
@@ -1687,22 +1739,22 @@
       <c r="G15" s="2"/>
       <c r="H15" s="2"/>
       <c r="I15" s="2" t="s">
-        <v>96</v>
+        <v>99</v>
       </c>
       <c r="J15" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O15" s="2" t="n">
         <v>0</v>
@@ -1720,24 +1772,27 @@
         <v>1</v>
       </c>
       <c r="T15" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U15" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
+        <v>101</v>
+      </c>
+      <c r="B16" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E16" s="2" t="s">
         <v>98</v>
-      </c>
-      <c r="B16" s="2" t="s">
-        <v>99</v>
-      </c>
-      <c r="C16" s="2" t="s">
-        <v>100</v>
-      </c>
-      <c r="D16" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="E16" s="2" t="s">
-        <v>95</v>
       </c>
       <c r="F16" s="2" t="n">
         <v>2024</v>
@@ -1745,22 +1800,22 @@
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2" t="s">
-        <v>101</v>
+        <v>104</v>
       </c>
       <c r="J16" s="2" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>102</v>
+        <v>105</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="O16" s="2"/>
       <c r="P16" s="2" t="n">
@@ -1776,7 +1831,10 @@
         <v>1</v>
       </c>
       <c r="T16" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U16" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>
@@ -1809,7 +1867,8 @@
     <col min="17" max="17" width="17.71" hidden="0" customWidth="1"/>
     <col min="18" max="18" width="18.71" hidden="0" customWidth="1"/>
     <col min="19" max="19" width="16.71" hidden="0" customWidth="1"/>
-    <col min="20" max="20" width="8.71" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="18.71" hidden="0" customWidth="1"/>
+    <col min="21" max="21" width="8.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1873,42 +1932,47 @@
       <c r="T1" s="2" t="s">
         <v>19</v>
       </c>
+      <c r="U1" s="2" t="s">
+        <v>20</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>103</v>
+        <v>106</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>104</v>
+        <v>107</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>105</v>
+        <v>108</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F2" s="2" t="n">
         <v>2027</v>
       </c>
-      <c r="G2" s="2"/>
+      <c r="G2" s="2" t="n">
+        <v>44916</v>
+      </c>
       <c r="H2" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I2" s="2" t="s">
-        <v>108</v>
+        <v>111</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K2" s="2"/>
       <c r="L2" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="N2" s="2"/>
       <c r="O2" s="2"/>
@@ -1925,44 +1989,49 @@
         <v>1</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U2" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>111</v>
+        <v>114</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>112</v>
+        <v>115</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>113</v>
+        <v>116</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>106</v>
+        <v>109</v>
       </c>
       <c r="F3" s="2" t="n">
         <v>2027</v>
       </c>
-      <c r="G3" s="2"/>
+      <c r="G3" s="2" t="n">
+        <v>45273</v>
+      </c>
       <c r="H3" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I3" s="2" t="s">
-        <v>115</v>
+        <v>118</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K3" s="2"/>
       <c r="L3" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M3" s="2" t="s">
-        <v>110</v>
+        <v>113</v>
       </c>
       <c r="N3" s="2"/>
       <c r="O3" s="2"/>
@@ -1979,44 +2048,49 @@
         <v>0</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U3" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>116</v>
+        <v>119</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F4" s="2" t="n">
         <v>2028</v>
       </c>
-      <c r="G4" s="2"/>
+      <c r="G4" s="2" t="n">
+        <v>44964</v>
+      </c>
       <c r="H4" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I4" s="2" t="s">
-        <v>119</v>
+        <v>122</v>
       </c>
       <c r="J4" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K4" s="2"/>
       <c r="L4" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>120</v>
+        <v>123</v>
       </c>
       <c r="N4" s="2"/>
       <c r="O4" s="2"/>
@@ -2033,44 +2107,49 @@
         <v>0</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U4" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>121</v>
+        <v>124</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F5" s="2" t="n">
         <v>2028</v>
       </c>
-      <c r="G5" s="2"/>
+      <c r="G5" s="2" t="n">
+        <v>44816</v>
+      </c>
       <c r="H5" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I5" s="2" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K5" s="2"/>
       <c r="L5" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="N5" s="2"/>
       <c r="O5" s="2"/>
@@ -2087,24 +2166,27 @@
         <v>0</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U5" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="F6" s="2" t="n">
         <v>2018</v>
@@ -2112,17 +2194,17 @@
       <c r="G6" s="2"/>
       <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K6" s="2"/>
       <c r="L6" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
@@ -2139,44 +2221,49 @@
         <v>0</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U6" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>133</v>
+        <v>136</v>
       </c>
       <c r="D7" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="F7" s="2" t="n">
         <v>2027</v>
       </c>
-      <c r="G7" s="2"/>
+      <c r="G7" s="2" t="n">
+        <v>44974</v>
+      </c>
       <c r="H7" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K7" s="2"/>
       <c r="L7" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
@@ -2193,42 +2280,47 @@
         <v>1</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U7" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="G8" s="2"/>
+      <c r="G8" s="2" t="n">
+        <v>45243</v>
+      </c>
       <c r="H8" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K8" s="2"/>
       <c r="L8" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
@@ -2245,42 +2337,47 @@
         <v>0</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U8" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="C9" s="2"/>
       <c r="D9" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>2027</v>
       </c>
-      <c r="G9" s="2"/>
+      <c r="G9" s="2" t="n">
+        <v>45320</v>
+      </c>
       <c r="H9" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K9" s="2"/>
       <c r="L9" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
@@ -2297,44 +2394,49 @@
         <v>0</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U9" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>2027</v>
       </c>
-      <c r="G10" s="2"/>
+      <c r="G10" s="2" t="n">
+        <v>45211</v>
+      </c>
       <c r="H10" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K10" s="2"/>
       <c r="L10" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>76</v>
+        <v>79</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
@@ -2351,42 +2453,47 @@
         <v>0</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U10" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F11" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="G11" s="2"/>
+      <c r="G11" s="2" t="n">
+        <v>45345</v>
+      </c>
       <c r="H11" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K11" s="2"/>
       <c r="L11" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -2403,42 +2510,47 @@
         <v>0</v>
       </c>
       <c r="T11" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U11" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="C12" s="2"/>
       <c r="D12" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="F12" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="G12" s="2"/>
+      <c r="G12" s="2" t="n">
+        <v>45245</v>
+      </c>
       <c r="H12" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K12" s="2"/>
       <c r="L12" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
@@ -2455,24 +2567,27 @@
         <v>0</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U12" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>2027</v>
@@ -2481,20 +2596,20 @@
         <v>45937</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K13" s="2"/>
       <c r="L13" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
@@ -2511,42 +2626,47 @@
         <v>0</v>
       </c>
       <c r="T13" s="2" t="s">
-        <v>31</v>
+        <v>73</v>
+      </c>
+      <c r="U13" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="C14" s="2"/>
       <c r="D14" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>95</v>
+        <v>98</v>
       </c>
       <c r="F14" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="G14" s="2"/>
+      <c r="G14" s="2" t="n">
+        <v>45250</v>
+      </c>
       <c r="H14" s="2" t="s">
-        <v>114</v>
+        <v>117</v>
       </c>
       <c r="I14" s="2" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="J14" s="2" t="s">
-        <v>109</v>
+        <v>112</v>
       </c>
       <c r="K14" s="2"/>
       <c r="L14" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
@@ -2563,7 +2683,10 @@
         <v>0</v>
       </c>
       <c r="T14" s="2" t="s">
-        <v>31</v>
+        <v>32</v>
+      </c>
+      <c r="U14" s="2" t="s">
+        <v>33</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fix approval dates for ASAs
</commit_message>
<xml_diff>
--- a/inst/extdata/wb_projects_gov_afe.xlsx
+++ b/inst/extdata/wb_projects_gov_afe.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="158">
   <si>
     <t xml:space="preserve">proj_id</t>
   </si>
@@ -33,7 +33,7 @@
     <t xml:space="preserve">proj_approval_fy</t>
   </si>
   <si>
-    <t xml:space="preserve">asa_cn_approval_date</t>
+    <t xml:space="preserve">asa_approval_date</t>
   </si>
   <si>
     <t xml:space="preserve">task_type</t>
@@ -397,24 +397,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://opswork.worldbank.org/home/P179174</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P158914</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIME_SZ_Planning/Auditing_Medication</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The objective of this program is to increase the use of rigorous impact evaluation (IE) by governments and other stakeholders for knowledge generation and evidence-based policy formulation across sectors and countries. The program is part of the ?Impact Evaluation to Development Impact (i2i)? trust fund, which is supported by DFID and administered by the World Bank?s Development Impact Evaluation group (DECIE). More specifically, this program supports the following three activities: (i) financial support to new and ongoing IEs that contribute to improving the design and implementation of development policies through knowledge generation across themes such as agriculture and rural development, financial sector development, private sector development, labor markets, infrastructure, governance, climate change, gender, and fragile and conflict situations, among others; (ii) financial support for a select set of IEs for data collection; and (iii) technical assistance to IE task teams to ensure high quality of research products.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kingdom of Eswatini</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://opswork.worldbank.org/home/P158914</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jurgen Rene Blum (ADM)</t>
   </si>
   <si>
     <t xml:space="preserve">P179680</t>
@@ -850,7 +832,7 @@
     <col min="4" max="4" width="27.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="27.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="16.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="20.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="17.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="9.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="42.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="17.71" hidden="0" customWidth="1"/>
@@ -1854,7 +1836,7 @@
     <col min="4" max="4" width="27.71" hidden="0" customWidth="1"/>
     <col min="5" max="5" width="39.71" hidden="0" customWidth="1"/>
     <col min="6" max="6" width="16.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="20.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="17.71" hidden="0" customWidth="1"/>
     <col min="8" max="8" width="10.71" hidden="0" customWidth="1"/>
     <col min="9" max="9" width="42.71" hidden="0" customWidth="1"/>
     <col min="10" max="10" width="40.71" hidden="0" customWidth="1"/>
@@ -1989,7 +1971,7 @@
         <v>1</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="U2" s="2" t="s">
         <v>33</v>
@@ -2048,7 +2030,7 @@
         <v>0</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="U3" s="2" t="s">
         <v>33</v>
@@ -2107,7 +2089,7 @@
         <v>0</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="U4" s="2" t="s">
         <v>33</v>
@@ -2166,7 +2148,7 @@
         <v>0</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="U5" s="2" t="s">
         <v>33</v>
@@ -2186,15 +2168,19 @@
         <v>24</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>2027</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>44974</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>131</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>2018</v>
-      </c>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2" t="s">
-        <v>132</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>112</v>
@@ -2204,24 +2190,24 @@
         <v>29</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>133</v>
+        <v>57</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
       <c r="P6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T6" s="2" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="U6" s="2" t="s">
         <v>33</v>
@@ -2229,31 +2215,29 @@
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>136</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="C7" s="2"/>
       <c r="D7" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>44974</v>
+        <v>45243</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>110</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>112</v>
@@ -2263,24 +2247,24 @@
         <v>29</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
       <c r="P7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="U7" s="2" t="s">
         <v>33</v>
@@ -2288,29 +2272,29 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>45243</v>
+        <v>45320</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>110</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>112</v>
@@ -2320,24 +2304,24 @@
         <v>29</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
       <c r="P8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="U8" s="2" t="s">
         <v>33</v>
@@ -2345,29 +2329,31 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="C9" s="2"/>
+        <v>139</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>140</v>
+      </c>
       <c r="D9" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>2027</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>45320</v>
+        <v>45211</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>112</v>
@@ -2377,7 +2363,7 @@
         <v>29</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
@@ -2394,7 +2380,7 @@
         <v>0</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="U9" s="2" t="s">
         <v>33</v>
@@ -2402,31 +2388,29 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>146</v>
-      </c>
+        <v>143</v>
+      </c>
+      <c r="C10" s="2"/>
       <c r="D10" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>45211</v>
+        <v>45345</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>117</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>112</v>
@@ -2436,24 +2420,24 @@
         <v>29</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>79</v>
+        <v>145</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
       <c r="P10" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R10" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="U10" s="2" t="s">
         <v>33</v>
@@ -2461,29 +2445,29 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F11" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>45345</v>
+        <v>45245</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>117</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>112</v>
@@ -2493,7 +2477,7 @@
         <v>29</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>151</v>
+        <v>95</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -2510,7 +2494,7 @@
         <v>0</v>
       </c>
       <c r="T11" s="2" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="U11" s="2" t="s">
         <v>33</v>
@@ -2518,29 +2502,31 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C12" s="2"/>
+        <v>150</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>151</v>
+      </c>
       <c r="D12" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>93</v>
+        <v>152</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>2026</v>
+        <v>2027</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>45245</v>
+        <v>45937</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>112</v>
@@ -2550,12 +2536,12 @@
         <v>29</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>95</v>
+        <v>154</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
       <c r="P12" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q12" s="2" t="n">
         <v>0</v>
@@ -2567,7 +2553,7 @@
         <v>0</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="U12" s="2" t="s">
         <v>33</v>
@@ -2580,26 +2566,24 @@
       <c r="B13" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>157</v>
-      </c>
+      <c r="C13" s="2"/>
       <c r="D13" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>158</v>
+        <v>98</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>2027</v>
+        <v>2026</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>45937</v>
+        <v>45250</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>112</v>
@@ -2609,12 +2593,12 @@
         <v>29</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>160</v>
+        <v>95</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
       <c r="P13" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="2" t="n">
         <v>0</v>
@@ -2629,63 +2613,6 @@
         <v>73</v>
       </c>
       <c r="U13" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>2026</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>45250</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U14" s="2" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>

<commit_message>
exclude asas missing approval fy
</commit_message>
<xml_diff>
--- a/inst/extdata/wb_projects_gov_afe.xlsx
+++ b/inst/extdata/wb_projects_gov_afe.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="164">
   <si>
     <t xml:space="preserve">proj_id</t>
   </si>
@@ -397,6 +397,24 @@
   </si>
   <si>
     <t xml:space="preserve">https://opswork.worldbank.org/home/P179174</t>
+  </si>
+  <si>
+    <t xml:space="preserve">P158914</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DIME_SZ_Planning/Auditing_Medication</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The objective of this program is to increase the use of rigorous impact evaluation (IE) by governments and other stakeholders for knowledge generation and evidence-based policy formulation across sectors and countries. The program is part of the ?Impact Evaluation to Development Impact (i2i)? trust fund, which is supported by DFID and administered by the World Bank?s Development Impact Evaluation group (DECIE). More specifically, this program supports the following three activities: (i) financial support to new and ongoing IEs that contribute to improving the design and implementation of development policies through knowledge generation across themes such as agriculture and rural development, financial sector development, private sector development, labor markets, infrastructure, governance, climate change, gender, and fragile and conflict situations, among others; (ii) financial support for a select set of IEs for data collection; and (iii) technical assistance to IE task teams to ensure high quality of research products.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Kingdom of Eswatini</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://opswork.worldbank.org/home/P158914</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Jurgen Rene Blum (ADM)</t>
   </si>
   <si>
     <t xml:space="preserve">P179680</t>
@@ -1935,7 +1953,7 @@
         <v>109</v>
       </c>
       <c r="F2" s="2" t="n">
-        <v>2027</v>
+        <v>2023</v>
       </c>
       <c r="G2" s="2" t="n">
         <v>44916</v>
@@ -1971,7 +1989,7 @@
         <v>1</v>
       </c>
       <c r="T2" s="2" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="U2" s="2" t="s">
         <v>33</v>
@@ -1994,7 +2012,7 @@
         <v>109</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>2027</v>
+        <v>2024</v>
       </c>
       <c r="G3" s="2" t="n">
         <v>45273</v>
@@ -2030,7 +2048,7 @@
         <v>0</v>
       </c>
       <c r="T3" s="2" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="U3" s="2" t="s">
         <v>33</v>
@@ -2053,7 +2071,7 @@
         <v>25</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>2028</v>
+        <v>2023</v>
       </c>
       <c r="G4" s="2" t="n">
         <v>44964</v>
@@ -2089,7 +2107,7 @@
         <v>0</v>
       </c>
       <c r="T4" s="2" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="U4" s="2" t="s">
         <v>33</v>
@@ -2112,7 +2130,7 @@
         <v>25</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>2028</v>
+        <v>2023</v>
       </c>
       <c r="G5" s="2" t="n">
         <v>44816</v>
@@ -2148,7 +2166,7 @@
         <v>0</v>
       </c>
       <c r="T5" s="2" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="U5" s="2" t="s">
         <v>33</v>
@@ -2168,19 +2186,13 @@
         <v>24</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F6" s="2" t="n">
-        <v>2027</v>
-      </c>
-      <c r="G6" s="2" t="n">
-        <v>44974</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>110</v>
-      </c>
+        <v>131</v>
+      </c>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+      <c r="H6" s="2"/>
       <c r="I6" s="2" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>112</v>
@@ -2190,54 +2202,54 @@
         <v>29</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>57</v>
+        <v>133</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
       <c r="P6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T6" s="2" t="s">
-        <v>73</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="T6" s="2"/>
       <c r="U6" s="2" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>133</v>
-      </c>
-      <c r="C7" s="2"/>
+        <v>135</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>136</v>
+      </c>
       <c r="D7" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>61</v>
+        <v>49</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>2026</v>
+        <v>2023</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>45243</v>
+        <v>44974</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>110</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>134</v>
+        <v>137</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>112</v>
@@ -2247,24 +2259,24 @@
         <v>29</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>63</v>
+        <v>57</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
       <c r="P7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T7" s="2" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="U7" s="2" t="s">
         <v>33</v>
@@ -2272,29 +2284,29 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>70</v>
+        <v>61</v>
       </c>
       <c r="F8" s="2" t="n">
-        <v>2027</v>
+        <v>2024</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>45320</v>
+        <v>45243</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>110</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>112</v>
@@ -2304,24 +2316,24 @@
         <v>29</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>72</v>
+        <v>63</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
       <c r="P8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="T8" s="2" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="U8" s="2" t="s">
         <v>33</v>
@@ -2329,31 +2341,29 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>139</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>140</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="C9" s="2"/>
       <c r="D9" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>77</v>
+        <v>70</v>
       </c>
       <c r="F9" s="2" t="n">
-        <v>2027</v>
+        <v>2024</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>45211</v>
+        <v>45320</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>112</v>
@@ -2363,7 +2373,7 @@
         <v>29</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>79</v>
+        <v>72</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
@@ -2380,7 +2390,7 @@
         <v>0</v>
       </c>
       <c r="T9" s="2" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="U9" s="2" t="s">
         <v>33</v>
@@ -2388,29 +2398,31 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>143</v>
-      </c>
-      <c r="C10" s="2"/>
+        <v>145</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>146</v>
+      </c>
       <c r="D10" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>87</v>
+        <v>77</v>
       </c>
       <c r="F10" s="2" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>45345</v>
+        <v>45211</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>117</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>112</v>
@@ -2420,24 +2432,24 @@
         <v>29</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>145</v>
+        <v>79</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
       <c r="P10" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R10" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="U10" s="2" t="s">
         <v>33</v>
@@ -2445,29 +2457,29 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>93</v>
+        <v>87</v>
       </c>
       <c r="F11" s="2" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>45245</v>
+        <v>45345</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>117</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>112</v>
@@ -2477,7 +2489,7 @@
         <v>29</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>95</v>
+        <v>151</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -2494,7 +2506,7 @@
         <v>0</v>
       </c>
       <c r="T11" s="2" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="U11" s="2" t="s">
         <v>33</v>
@@ -2502,31 +2514,29 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>150</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>151</v>
-      </c>
+        <v>153</v>
+      </c>
+      <c r="C12" s="2"/>
       <c r="D12" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>152</v>
+        <v>93</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>2027</v>
+        <v>2024</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>45937</v>
+        <v>45245</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>112</v>
@@ -2536,12 +2546,12 @@
         <v>29</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>154</v>
+        <v>95</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
       <c r="P12" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q12" s="2" t="n">
         <v>0</v>
@@ -2553,7 +2563,7 @@
         <v>0</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="U12" s="2" t="s">
         <v>33</v>
@@ -2566,24 +2576,26 @@
       <c r="B13" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="C13" s="2"/>
+      <c r="C13" s="2" t="s">
+        <v>157</v>
+      </c>
       <c r="D13" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>98</v>
+        <v>158</v>
       </c>
       <c r="F13" s="2" t="n">
         <v>2026</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>45250</v>
+        <v>45937</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>112</v>
@@ -2593,12 +2605,12 @@
         <v>29</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>95</v>
+        <v>160</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
       <c r="P13" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q13" s="2" t="n">
         <v>0</v>
@@ -2613,6 +2625,63 @@
         <v>73</v>
       </c>
       <c r="U13" s="2" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="s">
+        <v>161</v>
+      </c>
+      <c r="B14" s="2" t="s">
+        <v>162</v>
+      </c>
+      <c r="C14" s="2"/>
+      <c r="D14" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>98</v>
+      </c>
+      <c r="F14" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="G14" s="2" t="n">
+        <v>45250</v>
+      </c>
+      <c r="H14" s="2" t="s">
+        <v>117</v>
+      </c>
+      <c r="I14" s="2" t="s">
+        <v>163</v>
+      </c>
+      <c r="J14" s="2" t="s">
+        <v>112</v>
+      </c>
+      <c r="K14" s="2"/>
+      <c r="L14" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="M14" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="N14" s="2"/>
+      <c r="O14" s="2"/>
+      <c r="P14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="R14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S14" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="T14" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="U14" s="2" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>

<commit_message>
fix data pipeline for ASAs
</commit_message>
<xml_diff>
--- a/inst/extdata/wb_projects_gov_afe.xlsx
+++ b/inst/extdata/wb_projects_gov_afe.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="164">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="158">
   <si>
     <t xml:space="preserve">proj_id</t>
   </si>
@@ -397,24 +397,6 @@
   </si>
   <si>
     <t xml:space="preserve">https://opswork.worldbank.org/home/P179174</t>
-  </si>
-  <si>
-    <t xml:space="preserve">P158914</t>
-  </si>
-  <si>
-    <t xml:space="preserve">DIME_SZ_Planning/Auditing_Medication</t>
-  </si>
-  <si>
-    <t xml:space="preserve">The objective of this program is to increase the use of rigorous impact evaluation (IE) by governments and other stakeholders for knowledge generation and evidence-based policy formulation across sectors and countries. The program is part of the ?Impact Evaluation to Development Impact (i2i)? trust fund, which is supported by DFID and administered by the World Bank?s Development Impact Evaluation group (DECIE). More specifically, this program supports the following three activities: (i) financial support to new and ongoing IEs that contribute to improving the design and implementation of development policies through knowledge generation across themes such as agriculture and rural development, financial sector development, private sector development, labor markets, infrastructure, governance, climate change, gender, and fragile and conflict situations, among others; (ii) financial support for a select set of IEs for data collection; and (iii) technical assistance to IE task teams to ensure high quality of research products.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Kingdom of Eswatini</t>
-  </si>
-  <si>
-    <t xml:space="preserve">https://opswork.worldbank.org/home/P158914</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Jurgen Rene Blum (ADM)</t>
   </si>
   <si>
     <t xml:space="preserve">P179680</t>
@@ -2186,13 +2168,19 @@
         <v>24</v>
       </c>
       <c r="E6" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F6" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="G6" s="2" t="n">
+        <v>44974</v>
+      </c>
+      <c r="H6" s="2" t="s">
+        <v>110</v>
+      </c>
+      <c r="I6" s="2" t="s">
         <v>131</v>
-      </c>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
-      <c r="I6" s="2" t="s">
-        <v>132</v>
       </c>
       <c r="J6" s="2" t="s">
         <v>112</v>
@@ -2202,54 +2190,54 @@
         <v>29</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>133</v>
+        <v>57</v>
       </c>
       <c r="N6" s="2"/>
       <c r="O6" s="2"/>
       <c r="P6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q6" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S6" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" s="2"/>
+        <v>1</v>
+      </c>
+      <c r="T6" s="2" t="s">
+        <v>32</v>
+      </c>
       <c r="U6" s="2" t="s">
         <v>33</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>135</v>
-      </c>
-      <c r="C7" s="2" t="s">
-        <v>136</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="C7" s="2"/>
       <c r="D7" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>49</v>
+        <v>61</v>
       </c>
       <c r="F7" s="2" t="n">
-        <v>2023</v>
+        <v>2024</v>
       </c>
       <c r="G7" s="2" t="n">
-        <v>44974</v>
+        <v>45243</v>
       </c>
       <c r="H7" s="2" t="s">
         <v>110</v>
       </c>
       <c r="I7" s="2" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="J7" s="2" t="s">
         <v>112</v>
@@ -2259,21 +2247,21 @@
         <v>29</v>
       </c>
       <c r="M7" s="2" t="s">
-        <v>57</v>
+        <v>63</v>
       </c>
       <c r="N7" s="2"/>
       <c r="O7" s="2"/>
       <c r="P7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q7" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="T7" s="2" t="s">
         <v>32</v>
@@ -2284,29 +2272,29 @@
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="F8" s="2" t="n">
         <v>2024</v>
       </c>
       <c r="G8" s="2" t="n">
-        <v>45243</v>
+        <v>45320</v>
       </c>
       <c r="H8" s="2" t="s">
         <v>110</v>
       </c>
       <c r="I8" s="2" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="J8" s="2" t="s">
         <v>112</v>
@@ -2316,18 +2304,18 @@
         <v>29</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="N8" s="2"/>
       <c r="O8" s="2"/>
       <c r="P8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>0</v>
@@ -2341,29 +2329,31 @@
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>142</v>
-      </c>
-      <c r="C9" s="2"/>
+        <v>139</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>140</v>
+      </c>
       <c r="D9" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>70</v>
+        <v>77</v>
       </c>
       <c r="F9" s="2" t="n">
         <v>2024</v>
       </c>
       <c r="G9" s="2" t="n">
-        <v>45320</v>
+        <v>45211</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="I9" s="2" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="J9" s="2" t="s">
         <v>112</v>
@@ -2373,7 +2363,7 @@
         <v>29</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>72</v>
+        <v>79</v>
       </c>
       <c r="N9" s="2"/>
       <c r="O9" s="2"/>
@@ -2398,31 +2388,29 @@
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="C10" s="2" t="s">
-        <v>146</v>
-      </c>
+        <v>143</v>
+      </c>
+      <c r="C10" s="2"/>
       <c r="D10" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>77</v>
+        <v>87</v>
       </c>
       <c r="F10" s="2" t="n">
         <v>2024</v>
       </c>
       <c r="G10" s="2" t="n">
-        <v>45211</v>
+        <v>45345</v>
       </c>
       <c r="H10" s="2" t="s">
         <v>117</v>
       </c>
       <c r="I10" s="2" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="J10" s="2" t="s">
         <v>112</v>
@@ -2432,18 +2420,18 @@
         <v>29</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>79</v>
+        <v>145</v>
       </c>
       <c r="N10" s="2"/>
       <c r="O10" s="2"/>
       <c r="P10" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q10" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R10" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S10" s="2" t="n">
         <v>0</v>
@@ -2457,29 +2445,29 @@
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>87</v>
+        <v>93</v>
       </c>
       <c r="F11" s="2" t="n">
         <v>2024</v>
       </c>
       <c r="G11" s="2" t="n">
-        <v>45345</v>
+        <v>45245</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>117</v>
       </c>
       <c r="I11" s="2" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="J11" s="2" t="s">
         <v>112</v>
@@ -2489,7 +2477,7 @@
         <v>29</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>151</v>
+        <v>95</v>
       </c>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -2514,29 +2502,31 @@
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>153</v>
-      </c>
-      <c r="C12" s="2"/>
+        <v>150</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>151</v>
+      </c>
       <c r="D12" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>93</v>
+        <v>152</v>
       </c>
       <c r="F12" s="2" t="n">
-        <v>2024</v>
+        <v>2026</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>45245</v>
+        <v>45937</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>117</v>
+        <v>110</v>
       </c>
       <c r="I12" s="2" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="J12" s="2" t="s">
         <v>112</v>
@@ -2546,12 +2536,12 @@
         <v>29</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>95</v>
+        <v>154</v>
       </c>
       <c r="N12" s="2"/>
       <c r="O12" s="2"/>
       <c r="P12" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q12" s="2" t="n">
         <v>0</v>
@@ -2563,7 +2553,7 @@
         <v>0</v>
       </c>
       <c r="T12" s="2" t="s">
-        <v>32</v>
+        <v>73</v>
       </c>
       <c r="U12" s="2" t="s">
         <v>33</v>
@@ -2576,26 +2566,24 @@
       <c r="B13" s="2" t="s">
         <v>156</v>
       </c>
-      <c r="C13" s="2" t="s">
-        <v>157</v>
-      </c>
+      <c r="C13" s="2"/>
       <c r="D13" s="2" t="s">
         <v>24</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>158</v>
+        <v>98</v>
       </c>
       <c r="F13" s="2" t="n">
-        <v>2026</v>
+        <v>2024</v>
       </c>
       <c r="G13" s="2" t="n">
-        <v>45937</v>
+        <v>45250</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>110</v>
+        <v>117</v>
       </c>
       <c r="I13" s="2" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="J13" s="2" t="s">
         <v>112</v>
@@ -2605,12 +2593,12 @@
         <v>29</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>160</v>
+        <v>95</v>
       </c>
       <c r="N13" s="2"/>
       <c r="O13" s="2"/>
       <c r="P13" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q13" s="2" t="n">
         <v>0</v>
@@ -2622,66 +2610,9 @@
         <v>0</v>
       </c>
       <c r="T13" s="2" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="U13" s="2" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="2" t="s">
-        <v>161</v>
-      </c>
-      <c r="B14" s="2" t="s">
-        <v>162</v>
-      </c>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>45250</v>
-      </c>
-      <c r="H14" s="2" t="s">
-        <v>117</v>
-      </c>
-      <c r="I14" s="2" t="s">
-        <v>163</v>
-      </c>
-      <c r="J14" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="M14" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="N14" s="2"/>
-      <c r="O14" s="2"/>
-      <c r="P14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U14" s="2" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>

<commit_message>
add country_code to wb_projects_gov
</commit_message>
<xml_diff>
--- a/inst/extdata/wb_projects_gov_afe.xlsx
+++ b/inst/extdata/wb_projects_gov_afe.xlsx
@@ -13,7 +13,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="158" uniqueCount="158">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="170" uniqueCount="170">
   <si>
     <t xml:space="preserve">proj_id</t>
   </si>
@@ -27,6 +27,9 @@
     <t xml:space="preserve">region</t>
   </si>
   <si>
+    <t xml:space="preserve">country_code</t>
+  </si>
+  <si>
     <t xml:space="preserve">country_name</t>
   </si>
   <si>
@@ -90,6 +93,9 @@
     <t xml:space="preserve">Eastern and Southern Africa</t>
   </si>
   <si>
+    <t xml:space="preserve">SOM</t>
+  </si>
+  <si>
     <t xml:space="preserve">Federal Republic of Somalia</t>
   </si>
   <si>
@@ -144,6 +150,9 @@
     <t xml:space="preserve">To strengthen expenditure controls  and increase the efficiency of selected administrative services.</t>
   </si>
   <si>
+    <t xml:space="preserve">LSO</t>
+  </si>
+  <si>
     <t xml:space="preserve">Kingdom of Lesotho</t>
   </si>
   <si>
@@ -162,6 +171,9 @@
     <t xml:space="preserve">To strengthen county performance in the financing, management, coordination, and accountability for resources</t>
   </si>
   <si>
+    <t xml:space="preserve">KEN</t>
+  </si>
+  <si>
     <t xml:space="preserve">Republic of Kenya</t>
   </si>
   <si>
@@ -198,6 +210,9 @@
     <t xml:space="preserve">The objective of the Project is to: (i) strengthen Local Authorities? institutional performance, responsiveness to citizens and management of resources for service delivery; and (ii) in case of an Eligible Crisis or Emergency, respond promptly and effectively to it.</t>
   </si>
   <si>
+    <t xml:space="preserve">MWI</t>
+  </si>
+  <si>
     <t xml:space="preserve">Republic of Malawi</t>
   </si>
   <si>
@@ -225,6 +240,9 @@
     <t xml:space="preserve">To enhance domestic revenue collection and improve the efficiency, transparency, and job creation potential of public spending</t>
   </si>
   <si>
+    <t xml:space="preserve">RWA</t>
+  </si>
+  <si>
     <t xml:space="preserve">Republic of Rwanda</t>
   </si>
   <si>
@@ -246,6 +264,9 @@
     <t xml:space="preserve">To improve and build capacity for budget preparation and implementation.</t>
   </si>
   <si>
+    <t xml:space="preserve">SSD</t>
+  </si>
+  <si>
     <t xml:space="preserve">Republic of South Sudan</t>
   </si>
   <si>
@@ -276,6 +297,9 @@
     <t xml:space="preserve">To strengthen the GoU's efficiency, accountability, and sustainability of public investment and asset management.</t>
   </si>
   <si>
+    <t xml:space="preserve">UGA</t>
+  </si>
+  <si>
     <t xml:space="preserve">Republic of Uganda</t>
   </si>
   <si>
@@ -294,6 +318,9 @@
     <t xml:space="preserve">To strengthen the financing, institutional performance and accountability of local authorities in Zambia.</t>
   </si>
   <si>
+    <t xml:space="preserve">ZMB</t>
+  </si>
+  <si>
     <t xml:space="preserve">Republic of Zambia</t>
   </si>
   <si>
@@ -309,6 +336,9 @@
     <t xml:space="preserve">Public Finance Management and Procurement Systems for Service Delivery Program</t>
   </si>
   <si>
+    <t xml:space="preserve">TZA</t>
+  </si>
+  <si>
     <t xml:space="preserve">United Republic of Tanzania</t>
   </si>
   <si>
@@ -342,6 +372,9 @@
     <t xml:space="preserve">23.  The development objective of this ASA is to support the GoE?s endeavors toward more capable and sustainable institutions for better service delivery, transparency, and accountability. 24. The proposed analytical products will help to inform planned WB operations. The WB is currently in the project preparation phase of a new governance operation to support governance modernization to enable fiscal sustainability and improved service delivery (P178808). Proposed diagnostic work under Pillar 1 is a continuation of ongoing support under the MDTF of the adoption of IFRs in Ethiopia for greater transparency and accountability, and of the development and implementation of an effective PIM for better outcome and fiscal sustainability. Additional diagnostics in the areas of civil service and digital governance will serve as an analytical foundation for the operation under preparation. Proposed diagnostic and TA work under Pillar 2 is closely aligned with forthcoming work on the development of Ethiopia?s Country Climate and Development Report (P179525), and in the case of the Governance GP, development of early tools to track CC related budgets, and reporting and to embed CC consideration in PIM reforms underway.</t>
   </si>
   <si>
+    <t xml:space="preserve">ETH</t>
+  </si>
+  <si>
     <t xml:space="preserve">Federal Democratic Republic of Ethiopia</t>
   </si>
   <si>
@@ -469,6 +502,9 @@
   </si>
   <si>
     <t xml:space="preserve">To advance institutional reforms in Zimbabwe?s public sector by strengthening the oversight and performance of State-Owned Enterprises (SOEs), enhancing public financial management (PFM) systems, and increasing access to justice, particularly for vulnerable and marginalized litigants.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZWE</t>
   </si>
   <si>
     <t xml:space="preserve">Republic of Zimbabwe</t>
@@ -830,23 +866,24 @@
     <col min="2" max="2" width="40.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="60.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="27.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="27.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="16.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="17.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="9.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="42.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="17.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="18.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="7.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="32.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="14.71" hidden="0" customWidth="1"/>
-    <col min="15" max="15" width="17.71" hidden="0" customWidth="1"/>
-    <col min="16" max="16" width="9.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="17.71" hidden="0" customWidth="1"/>
-    <col min="18" max="18" width="18.71" hidden="0" customWidth="1"/>
-    <col min="19" max="19" width="16.71" hidden="0" customWidth="1"/>
-    <col min="20" max="20" width="18.71" hidden="0" customWidth="1"/>
-    <col min="21" max="21" width="8.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="12.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="27.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="17.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="9.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="42.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="17.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="18.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="7.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="32.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="14.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="17.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="9.71" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="17.71" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="18.71" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="16.71" hidden="0" customWidth="1"/>
+    <col min="21" max="21" width="18.71" hidden="0" customWidth="1"/>
+    <col min="22" max="22" width="8.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -913,475 +950,499 @@
       <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
+      <c r="V1" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F2" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>2020</v>
       </c>
-      <c r="G2" s="2"/>
       <c r="H2" s="2"/>
-      <c r="I2" s="2" t="s">
-        <v>26</v>
-      </c>
+      <c r="I2" s="2"/>
       <c r="J2" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="K2" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L2" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M2" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N2" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O2" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="O2" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P2" s="2" t="n">
         <v>135000000</v>
       </c>
-      <c r="P2" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="Q2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T2" s="2" t="s">
-        <v>32</v>
+        <v>1</v>
+      </c>
+      <c r="T2" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="B3" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G3" s="2" t="n">
+        <v>2022</v>
+      </c>
+      <c r="H3" s="2"/>
+      <c r="I3" s="2"/>
+      <c r="J3" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="L3" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="M3" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="O3" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P3" s="2" t="n">
+        <v>62000000</v>
+      </c>
+      <c r="Q3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="R3" s="2" t="n">
+        <v>0</v>
+      </c>
+      <c r="S3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="T3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="U3" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="2" t="s">
+      <c r="V3" s="2" t="s">
         <v>35</v>
-      </c>
-      <c r="C3" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D3" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E3" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F3" s="2" t="n">
-        <v>2022</v>
-      </c>
-      <c r="G3" s="2"/>
-      <c r="H3" s="2"/>
-      <c r="I3" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="J3" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K3" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="L3" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="M3" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="N3" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O3" s="2" t="n">
-        <v>62000000</v>
-      </c>
-      <c r="P3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="Q3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="R3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="S3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T3" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="U3" s="2" t="s">
-        <v>33</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="G4" s="2"/>
       <c r="H4" s="2"/>
-      <c r="I4" s="2" t="s">
-        <v>39</v>
-      </c>
+      <c r="I4" s="2"/>
       <c r="J4" s="2" t="s">
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="K4" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L4" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M4" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="N4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O4" s="2" t="n">
-        <v>0</v>
+        <v>32</v>
+      </c>
+      <c r="O4" s="2" t="s">
+        <v>33</v>
       </c>
       <c r="P4" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q4" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R4" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T4" s="2" t="s">
-        <v>32</v>
+      <c r="T4" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="U4" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>43</v>
-      </c>
-      <c r="F5" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="G5" s="2"/>
       <c r="H5" s="2"/>
-      <c r="I5" s="2" t="s">
-        <v>44</v>
-      </c>
+      <c r="I5" s="2"/>
       <c r="J5" s="2" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="K5" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L5" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M5" s="2" t="s">
-        <v>45</v>
+        <v>31</v>
       </c>
       <c r="N5" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O5" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="O5" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P5" s="2" t="n">
         <v>20000000</v>
       </c>
-      <c r="P5" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="Q5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R5" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T5" s="2" t="s">
-        <v>32</v>
+      <c r="T5" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="U5" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V5" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F6" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="G6" s="2"/>
       <c r="H6" s="2"/>
-      <c r="I6" s="2" t="s">
-        <v>50</v>
-      </c>
+      <c r="I6" s="2"/>
       <c r="J6" s="2" t="s">
-        <v>27</v>
+        <v>54</v>
       </c>
       <c r="K6" s="2" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="L6" s="2" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="M6" s="2" t="s">
-        <v>52</v>
+        <v>31</v>
       </c>
       <c r="N6" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O6" s="2" t="n">
+        <v>56</v>
+      </c>
+      <c r="O6" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P6" s="2" t="n">
         <v>150000000</v>
       </c>
-      <c r="P6" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="Q6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T6" s="2" t="s">
-        <v>32</v>
+      <c r="T6" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="U6" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V6" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>59</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>52</v>
+      </c>
+      <c r="F7" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="B7" s="2" t="s">
-        <v>54</v>
-      </c>
-      <c r="C7" s="2" t="s">
+      <c r="G7" s="2" t="n">
+        <v>2024</v>
+      </c>
+      <c r="H7" s="2"/>
+      <c r="I7" s="2"/>
+      <c r="J7" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="L7" s="2" t="s">
         <v>55</v>
       </c>
-      <c r="D7" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E7" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>2024</v>
-      </c>
-      <c r="G7" s="2"/>
-      <c r="H7" s="2"/>
-      <c r="I7" s="2" t="s">
-        <v>56</v>
-      </c>
-      <c r="J7" s="2" t="s">
-        <v>27</v>
-      </c>
-      <c r="K7" s="2" t="s">
-        <v>51</v>
-      </c>
-      <c r="L7" s="2" t="s">
-        <v>29</v>
-      </c>
       <c r="M7" s="2" t="s">
-        <v>57</v>
+        <v>31</v>
       </c>
       <c r="N7" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O7" s="2" t="n">
+        <v>61</v>
+      </c>
+      <c r="O7" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P7" s="2" t="n">
         <v>200000000</v>
       </c>
-      <c r="P7" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="Q7" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R7" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T7" s="2" t="s">
-        <v>32</v>
+      <c r="T7" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="U7" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V7" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="D8" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F8" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G8" s="2" t="n">
         <v>2020</v>
       </c>
-      <c r="G8" s="2"/>
       <c r="H8" s="2"/>
-      <c r="I8" s="2" t="s">
-        <v>62</v>
-      </c>
+      <c r="I8" s="2"/>
       <c r="J8" s="2" t="s">
-        <v>27</v>
+        <v>67</v>
       </c>
       <c r="K8" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L8" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M8" s="2" t="s">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="N8" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O8" s="2" t="n">
+        <v>68</v>
+      </c>
+      <c r="O8" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P8" s="2" t="n">
         <v>100000000</v>
       </c>
-      <c r="P8" s="2" t="n">
-        <v>0</v>
-      </c>
       <c r="Q8" s="2" t="n">
         <v>0</v>
       </c>
       <c r="R8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S8" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T8" s="2" t="s">
-        <v>32</v>
+      <c r="T8" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="U8" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V8" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="C9" s="2" t="s">
         <v>64</v>
       </c>
-      <c r="B9" s="2" t="s">
+      <c r="D9" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="2" t="s">
         <v>65</v>
       </c>
-      <c r="C9" s="2" t="s">
-        <v>60</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F9" s="2" t="n">
+      <c r="F9" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="G9" s="2"/>
       <c r="H9" s="2"/>
-      <c r="I9" s="2" t="s">
-        <v>66</v>
-      </c>
+      <c r="I9" s="2"/>
       <c r="J9" s="2" t="s">
-        <v>27</v>
+        <v>71</v>
       </c>
       <c r="K9" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L9" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M9" s="2" t="s">
-        <v>63</v>
+        <v>31</v>
       </c>
       <c r="N9" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O9" s="2" t="n">
-        <v>0</v>
+        <v>68</v>
+      </c>
+      <c r="O9" s="2" t="s">
+        <v>33</v>
       </c>
       <c r="P9" s="2" t="n">
         <v>0</v>
@@ -1393,119 +1454,125 @@
         <v>0</v>
       </c>
       <c r="S9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T9" s="2" t="s">
-        <v>32</v>
+        <v>0</v>
+      </c>
+      <c r="T9" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="U9" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V9" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="F10" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="G10" s="2"/>
       <c r="H10" s="2"/>
-      <c r="I10" s="2" t="s">
-        <v>71</v>
-      </c>
+      <c r="I10" s="2"/>
       <c r="J10" s="2" t="s">
-        <v>27</v>
+        <v>77</v>
       </c>
       <c r="K10" s="2" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="L10" s="2" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>72</v>
+        <v>31</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O10" s="2"/>
-      <c r="P10" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>78</v>
+      </c>
+      <c r="O10" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P10" s="2"/>
       <c r="Q10" s="2" t="n">
         <v>1</v>
       </c>
       <c r="R10" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T10" s="2" t="s">
-        <v>73</v>
+        <v>0</v>
+      </c>
+      <c r="T10" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="U10" s="2" t="s">
-        <v>33</v>
+        <v>79</v>
+      </c>
+      <c r="V10" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="D11" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="F11" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="G11" s="2"/>
       <c r="H11" s="2"/>
-      <c r="I11" s="2" t="s">
-        <v>78</v>
-      </c>
+      <c r="I11" s="2"/>
       <c r="J11" s="2" t="s">
-        <v>27</v>
+        <v>85</v>
       </c>
       <c r="K11" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L11" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O11" s="2" t="n">
+        <v>86</v>
+      </c>
+      <c r="O11" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P11" s="2" t="n">
         <v>34000000</v>
       </c>
-      <c r="P11" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="Q11" s="2" t="n">
         <v>1</v>
       </c>
@@ -1513,58 +1580,61 @@
         <v>1</v>
       </c>
       <c r="S11" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" s="2" t="s">
-        <v>32</v>
+        <v>1</v>
+      </c>
+      <c r="T11" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="U11" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V11" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>80</v>
+        <v>87</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>81</v>
+        <v>88</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="F12" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>2025</v>
       </c>
-      <c r="G12" s="2"/>
       <c r="H12" s="2"/>
-      <c r="I12" s="2" t="s">
-        <v>83</v>
-      </c>
+      <c r="I12" s="2"/>
       <c r="J12" s="2" t="s">
-        <v>27</v>
+        <v>90</v>
       </c>
       <c r="K12" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L12" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M12" s="2" t="s">
-        <v>79</v>
+        <v>31</v>
       </c>
       <c r="N12" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O12" s="2"/>
-      <c r="P12" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>86</v>
+      </c>
+      <c r="O12" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P12" s="2"/>
       <c r="Q12" s="2" t="n">
         <v>0</v>
       </c>
@@ -1572,237 +1642,249 @@
         <v>0</v>
       </c>
       <c r="S12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T12" s="2" t="s">
-        <v>32</v>
+        <v>0</v>
+      </c>
+      <c r="T12" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="U12" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V12" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>84</v>
+        <v>91</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>85</v>
+        <v>92</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>86</v>
+        <v>93</v>
       </c>
       <c r="D13" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F13" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G13" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="G13" s="2"/>
       <c r="H13" s="2"/>
-      <c r="I13" s="2" t="s">
-        <v>88</v>
-      </c>
+      <c r="I13" s="2"/>
       <c r="J13" s="2" t="s">
-        <v>27</v>
+        <v>96</v>
       </c>
       <c r="K13" s="2" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="L13" s="2" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="M13" s="2" t="s">
-        <v>89</v>
+        <v>31</v>
       </c>
       <c r="N13" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O13" s="2"/>
-      <c r="P13" s="2" t="n">
-        <v>1</v>
-      </c>
+        <v>97</v>
+      </c>
+      <c r="O13" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P13" s="2"/>
       <c r="Q13" s="2" t="n">
         <v>1</v>
       </c>
       <c r="R13" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="S13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T13" s="2" t="s">
-        <v>73</v>
+        <v>0</v>
+      </c>
+      <c r="T13" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="U13" s="2" t="s">
-        <v>33</v>
+        <v>79</v>
+      </c>
+      <c r="V13" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="s">
-        <v>90</v>
+        <v>98</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>91</v>
+        <v>99</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>92</v>
+        <v>100</v>
       </c>
       <c r="D14" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E14" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="F14" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="F14" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="G14" s="2" t="n">
         <v>2022</v>
       </c>
-      <c r="G14" s="2"/>
       <c r="H14" s="2"/>
-      <c r="I14" s="2" t="s">
-        <v>94</v>
-      </c>
+      <c r="I14" s="2"/>
       <c r="J14" s="2" t="s">
-        <v>27</v>
+        <v>103</v>
       </c>
       <c r="K14" s="2" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="L14" s="2" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="M14" s="2" t="s">
-        <v>95</v>
+        <v>31</v>
       </c>
       <c r="N14" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O14" s="2" t="n">
+        <v>104</v>
+      </c>
+      <c r="O14" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P14" s="2" t="n">
         <v>210000000</v>
       </c>
-      <c r="P14" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="Q14" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R14" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T14" s="2" t="s">
-        <v>32</v>
+      <c r="T14" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="U14" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V14" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="C15" s="2"/>
       <c r="D15" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E15" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="F15" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="F15" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G15" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="G15" s="2"/>
       <c r="H15" s="2"/>
-      <c r="I15" s="2" t="s">
-        <v>99</v>
-      </c>
+      <c r="I15" s="2"/>
       <c r="J15" s="2" t="s">
-        <v>27</v>
+        <v>109</v>
       </c>
       <c r="K15" s="2" t="s">
-        <v>51</v>
+        <v>29</v>
       </c>
       <c r="L15" s="2" t="s">
-        <v>29</v>
+        <v>55</v>
       </c>
       <c r="M15" s="2" t="s">
-        <v>100</v>
+        <v>31</v>
       </c>
       <c r="N15" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O15" s="2" t="n">
-        <v>0</v>
+        <v>110</v>
+      </c>
+      <c r="O15" s="2" t="s">
+        <v>33</v>
       </c>
       <c r="P15" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q15" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R15" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T15" s="2" t="s">
-        <v>32</v>
+      <c r="T15" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="U15" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V15" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="s">
-        <v>101</v>
+        <v>111</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>102</v>
+        <v>112</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>103</v>
+        <v>113</v>
       </c>
       <c r="D16" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E16" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="F16" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="F16" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G16" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="G16" s="2"/>
       <c r="H16" s="2"/>
-      <c r="I16" s="2" t="s">
-        <v>104</v>
-      </c>
+      <c r="I16" s="2"/>
       <c r="J16" s="2" t="s">
-        <v>27</v>
+        <v>114</v>
       </c>
       <c r="K16" s="2" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="L16" s="2" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="M16" s="2" t="s">
-        <v>105</v>
+        <v>31</v>
       </c>
       <c r="N16" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O16" s="2"/>
-      <c r="P16" s="2" t="n">
-        <v>0</v>
-      </c>
+        <v>115</v>
+      </c>
+      <c r="O16" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="P16" s="2"/>
       <c r="Q16" s="2" t="n">
         <v>0</v>
       </c>
@@ -1810,13 +1892,16 @@
         <v>0</v>
       </c>
       <c r="S16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="T16" s="2" t="s">
-        <v>32</v>
+        <v>0</v>
+      </c>
+      <c r="T16" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="U16" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V16" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
@@ -1834,23 +1919,24 @@
     <col min="2" max="2" width="40.71" hidden="0" customWidth="1"/>
     <col min="3" max="3" width="60.71" hidden="0" customWidth="1"/>
     <col min="4" max="4" width="27.71" hidden="0" customWidth="1"/>
-    <col min="5" max="5" width="39.71" hidden="0" customWidth="1"/>
-    <col min="6" max="6" width="16.71" hidden="0" customWidth="1"/>
-    <col min="7" max="7" width="17.71" hidden="0" customWidth="1"/>
-    <col min="8" max="8" width="10.71" hidden="0" customWidth="1"/>
-    <col min="9" max="9" width="42.71" hidden="0" customWidth="1"/>
-    <col min="10" max="10" width="40.71" hidden="0" customWidth="1"/>
-    <col min="11" max="11" width="18.71" hidden="0" customWidth="1"/>
-    <col min="12" max="12" width="7.71" hidden="0" customWidth="1"/>
-    <col min="13" max="13" width="35.71" hidden="0" customWidth="1"/>
-    <col min="14" max="14" width="14.71" hidden="0" customWidth="1"/>
-    <col min="15" max="15" width="17.71" hidden="0" customWidth="1"/>
-    <col min="16" max="16" width="9.71" hidden="0" customWidth="1"/>
-    <col min="17" max="17" width="17.71" hidden="0" customWidth="1"/>
-    <col min="18" max="18" width="18.71" hidden="0" customWidth="1"/>
-    <col min="19" max="19" width="16.71" hidden="0" customWidth="1"/>
-    <col min="20" max="20" width="18.71" hidden="0" customWidth="1"/>
-    <col min="21" max="21" width="8.71" hidden="0" customWidth="1"/>
+    <col min="5" max="5" width="12.71" hidden="0" customWidth="1"/>
+    <col min="6" max="6" width="39.71" hidden="0" customWidth="1"/>
+    <col min="7" max="7" width="16.71" hidden="0" customWidth="1"/>
+    <col min="8" max="8" width="17.71" hidden="0" customWidth="1"/>
+    <col min="9" max="9" width="10.71" hidden="0" customWidth="1"/>
+    <col min="10" max="10" width="42.71" hidden="0" customWidth="1"/>
+    <col min="11" max="11" width="40.71" hidden="0" customWidth="1"/>
+    <col min="12" max="12" width="18.71" hidden="0" customWidth="1"/>
+    <col min="13" max="13" width="7.71" hidden="0" customWidth="1"/>
+    <col min="14" max="14" width="35.71" hidden="0" customWidth="1"/>
+    <col min="15" max="15" width="14.71" hidden="0" customWidth="1"/>
+    <col min="16" max="16" width="17.71" hidden="0" customWidth="1"/>
+    <col min="17" max="17" width="9.71" hidden="0" customWidth="1"/>
+    <col min="18" max="18" width="17.71" hidden="0" customWidth="1"/>
+    <col min="19" max="19" width="18.71" hidden="0" customWidth="1"/>
+    <col min="20" max="20" width="16.71" hidden="0" customWidth="1"/>
+    <col min="21" max="21" width="18.71" hidden="0" customWidth="1"/>
+    <col min="22" max="22" width="8.71" hidden="0" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1917,111 +2003,117 @@
       <c r="U1" s="2" t="s">
         <v>20</v>
       </c>
+      <c r="V1" s="2" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="s">
-        <v>106</v>
+        <v>116</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>107</v>
+        <v>117</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>108</v>
+        <v>118</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="F2" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G2" s="2" t="n">
         <v>2023</v>
       </c>
-      <c r="G2" s="2" t="n">
+      <c r="H2" s="2" t="n">
         <v>44916</v>
       </c>
-      <c r="H2" s="2" t="s">
-        <v>110</v>
-      </c>
       <c r="I2" s="2" t="s">
-        <v>111</v>
+        <v>121</v>
       </c>
       <c r="J2" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2" t="s">
-        <v>29</v>
-      </c>
+        <v>122</v>
+      </c>
+      <c r="K2" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="L2" s="2"/>
       <c r="M2" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="N2" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="N2" s="2" t="s">
+        <v>124</v>
+      </c>
       <c r="O2" s="2"/>
-      <c r="P2" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P2" s="2"/>
       <c r="Q2" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R2" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T2" s="2" t="s">
-        <v>32</v>
+      <c r="T2" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="U2" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V2" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="s">
-        <v>114</v>
+        <v>125</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>115</v>
+        <v>126</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>116</v>
+        <v>127</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>109</v>
-      </c>
-      <c r="F3" s="2" t="n">
+        <v>119</v>
+      </c>
+      <c r="F3" s="2" t="s">
+        <v>120</v>
+      </c>
+      <c r="G3" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="H3" s="2" t="n">
         <v>45273</v>
       </c>
-      <c r="H3" s="2" t="s">
-        <v>117</v>
-      </c>
       <c r="I3" s="2" t="s">
-        <v>118</v>
+        <v>128</v>
       </c>
       <c r="J3" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2" t="s">
-        <v>29</v>
-      </c>
+        <v>129</v>
+      </c>
+      <c r="K3" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="L3" s="2"/>
       <c r="M3" s="2" t="s">
-        <v>113</v>
-      </c>
-      <c r="N3" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="N3" s="2" t="s">
+        <v>124</v>
+      </c>
       <c r="O3" s="2"/>
-      <c r="P3" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P3" s="2"/>
       <c r="Q3" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R3" s="2" t="n">
         <v>0</v>
@@ -2029,117 +2121,123 @@
       <c r="S3" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T3" s="2" t="s">
-        <v>32</v>
+      <c r="T3" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="U3" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V3" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="s">
-        <v>119</v>
+        <v>130</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>120</v>
+        <v>131</v>
       </c>
       <c r="C4" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G4" s="2" t="n">
+        <v>2023</v>
+      </c>
+      <c r="H4" s="2" t="n">
+        <v>44964</v>
+      </c>
+      <c r="I4" s="2" t="s">
         <v>121</v>
       </c>
-      <c r="D4" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F4" s="2" t="n">
-        <v>2023</v>
-      </c>
-      <c r="G4" s="2" t="n">
-        <v>44964</v>
-      </c>
-      <c r="H4" s="2" t="s">
-        <v>110</v>
-      </c>
-      <c r="I4" s="2" t="s">
-        <v>122</v>
-      </c>
       <c r="J4" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2" t="s">
-        <v>29</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="K4" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="L4" s="2"/>
       <c r="M4" s="2" t="s">
-        <v>123</v>
-      </c>
-      <c r="N4" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="N4" s="2" t="s">
+        <v>134</v>
+      </c>
       <c r="O4" s="2"/>
-      <c r="P4" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P4" s="2"/>
       <c r="Q4" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R4" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S4" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T4" s="2" t="s">
-        <v>32</v>
+        <v>1</v>
+      </c>
+      <c r="T4" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="U4" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V4" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="s">
-        <v>124</v>
+        <v>135</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>125</v>
+        <v>136</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>126</v>
+        <v>137</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="F5" s="2" t="n">
+        <v>26</v>
+      </c>
+      <c r="F5" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="G5" s="2" t="n">
         <v>2023</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="H5" s="2" t="n">
         <v>44816</v>
       </c>
-      <c r="H5" s="2" t="s">
-        <v>110</v>
-      </c>
       <c r="I5" s="2" t="s">
-        <v>127</v>
+        <v>121</v>
       </c>
       <c r="J5" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2" t="s">
-        <v>29</v>
-      </c>
+        <v>138</v>
+      </c>
+      <c r="K5" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="L5" s="2"/>
       <c r="M5" s="2" t="s">
-        <v>89</v>
-      </c>
-      <c r="N5" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="N5" s="2" t="s">
+        <v>97</v>
+      </c>
       <c r="O5" s="2"/>
-      <c r="P5" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P5" s="2"/>
       <c r="Q5" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R5" s="2" t="n">
         <v>0</v>
@@ -2147,113 +2245,119 @@
       <c r="S5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T5" s="2" t="s">
-        <v>32</v>
+      <c r="T5" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="U5" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V5" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="s">
-        <v>128</v>
+        <v>139</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>129</v>
+        <v>140</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>130</v>
+        <v>141</v>
       </c>
       <c r="D6" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E6" s="2" t="s">
-        <v>49</v>
-      </c>
-      <c r="F6" s="2" t="n">
+        <v>52</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="G6" s="2" t="n">
         <v>2023</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="H6" s="2" t="n">
         <v>44974</v>
       </c>
-      <c r="H6" s="2" t="s">
-        <v>110</v>
-      </c>
       <c r="I6" s="2" t="s">
-        <v>131</v>
+        <v>121</v>
       </c>
       <c r="J6" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2" t="s">
-        <v>29</v>
-      </c>
+        <v>142</v>
+      </c>
+      <c r="K6" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="L6" s="2"/>
       <c r="M6" s="2" t="s">
-        <v>57</v>
-      </c>
-      <c r="N6" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="N6" s="2" t="s">
+        <v>61</v>
+      </c>
       <c r="O6" s="2"/>
-      <c r="P6" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P6" s="2"/>
       <c r="Q6" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R6" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="T6" s="2" t="s">
-        <v>32</v>
+      <c r="T6" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="U6" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V6" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="s">
-        <v>132</v>
+        <v>143</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>133</v>
+        <v>144</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E7" s="2" t="s">
-        <v>61</v>
-      </c>
-      <c r="F7" s="2" t="n">
+        <v>65</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>66</v>
+      </c>
+      <c r="G7" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="G7" s="2" t="n">
+      <c r="H7" s="2" t="n">
         <v>45243</v>
       </c>
-      <c r="H7" s="2" t="s">
-        <v>110</v>
-      </c>
       <c r="I7" s="2" t="s">
-        <v>134</v>
+        <v>121</v>
       </c>
       <c r="J7" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2" t="s">
-        <v>29</v>
-      </c>
+        <v>145</v>
+      </c>
+      <c r="K7" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="L7" s="2"/>
       <c r="M7" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="N7" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="N7" s="2" t="s">
+        <v>68</v>
+      </c>
       <c r="O7" s="2"/>
-      <c r="P7" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="P7" s="2"/>
       <c r="Q7" s="2" t="n">
         <v>0</v>
       </c>
@@ -2263,170 +2367,179 @@
       <c r="S7" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T7" s="2" t="s">
-        <v>32</v>
+      <c r="T7" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="U7" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V7" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="s">
-        <v>135</v>
+        <v>146</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>136</v>
+        <v>147</v>
       </c>
       <c r="C8" s="2"/>
       <c r="D8" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E8" s="2" t="s">
-        <v>70</v>
-      </c>
-      <c r="F8" s="2" t="n">
+        <v>75</v>
+      </c>
+      <c r="F8" s="2" t="s">
+        <v>76</v>
+      </c>
+      <c r="G8" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="G8" s="2" t="n">
+      <c r="H8" s="2" t="n">
         <v>45320</v>
       </c>
-      <c r="H8" s="2" t="s">
-        <v>110</v>
-      </c>
       <c r="I8" s="2" t="s">
-        <v>137</v>
+        <v>121</v>
       </c>
       <c r="J8" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2" t="s">
-        <v>29</v>
-      </c>
+        <v>148</v>
+      </c>
+      <c r="K8" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="L8" s="2"/>
       <c r="M8" s="2" t="s">
-        <v>72</v>
-      </c>
-      <c r="N8" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="N8" s="2" t="s">
+        <v>78</v>
+      </c>
       <c r="O8" s="2"/>
-      <c r="P8" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P8" s="2"/>
       <c r="Q8" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R8" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S8" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T8" s="2" t="s">
-        <v>32</v>
+        <v>1</v>
+      </c>
+      <c r="T8" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="U8" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V8" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="s">
-        <v>138</v>
+        <v>149</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>140</v>
+        <v>151</v>
       </c>
       <c r="D9" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E9" s="2" t="s">
-        <v>77</v>
-      </c>
-      <c r="F9" s="2" t="n">
+        <v>83</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="G9" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="G9" s="2" t="n">
+      <c r="H9" s="2" t="n">
         <v>45211</v>
       </c>
-      <c r="H9" s="2" t="s">
-        <v>117</v>
-      </c>
       <c r="I9" s="2" t="s">
-        <v>141</v>
+        <v>128</v>
       </c>
       <c r="J9" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2" t="s">
-        <v>29</v>
-      </c>
+        <v>152</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="L9" s="2"/>
       <c r="M9" s="2" t="s">
-        <v>79</v>
-      </c>
-      <c r="N9" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="N9" s="2" t="s">
+        <v>86</v>
+      </c>
       <c r="O9" s="2"/>
-      <c r="P9" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P9" s="2"/>
       <c r="Q9" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R9" s="2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="S9" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="T9" s="2" t="s">
-        <v>32</v>
+        <v>1</v>
+      </c>
+      <c r="T9" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="U9" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V9" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="s">
-        <v>142</v>
+        <v>153</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>143</v>
+        <v>154</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E10" s="2" t="s">
-        <v>87</v>
-      </c>
-      <c r="F10" s="2" t="n">
+        <v>94</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>95</v>
+      </c>
+      <c r="G10" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="G10" s="2" t="n">
+      <c r="H10" s="2" t="n">
         <v>45345</v>
       </c>
-      <c r="H10" s="2" t="s">
-        <v>117</v>
-      </c>
       <c r="I10" s="2" t="s">
-        <v>144</v>
+        <v>128</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2" t="s">
-        <v>29</v>
-      </c>
+        <v>155</v>
+      </c>
+      <c r="K10" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="L10" s="2"/>
       <c r="M10" s="2" t="s">
-        <v>145</v>
-      </c>
-      <c r="N10" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="N10" s="2" t="s">
+        <v>156</v>
+      </c>
       <c r="O10" s="2"/>
-      <c r="P10" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="P10" s="2"/>
       <c r="Q10" s="2" t="n">
         <v>0</v>
       </c>
@@ -2436,54 +2549,57 @@
       <c r="S10" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T10" s="2" t="s">
-        <v>32</v>
+      <c r="T10" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="U10" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V10" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="s">
-        <v>146</v>
+        <v>157</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>147</v>
+        <v>158</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E11" s="2" t="s">
-        <v>93</v>
-      </c>
-      <c r="F11" s="2" t="n">
+        <v>101</v>
+      </c>
+      <c r="F11" s="2" t="s">
+        <v>102</v>
+      </c>
+      <c r="G11" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="G11" s="2" t="n">
+      <c r="H11" s="2" t="n">
         <v>45245</v>
       </c>
-      <c r="H11" s="2" t="s">
-        <v>117</v>
-      </c>
       <c r="I11" s="2" t="s">
-        <v>148</v>
+        <v>128</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2" t="s">
-        <v>29</v>
-      </c>
+        <v>159</v>
+      </c>
+      <c r="K11" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="L11" s="2"/>
       <c r="M11" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="N11" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="N11" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="O11" s="2"/>
-      <c r="P11" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="P11" s="2"/>
       <c r="Q11" s="2" t="n">
         <v>0</v>
       </c>
@@ -2493,58 +2609,61 @@
       <c r="S11" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T11" s="2" t="s">
-        <v>32</v>
+      <c r="T11" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="U11" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V11" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="s">
-        <v>149</v>
+        <v>160</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>150</v>
+        <v>161</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>151</v>
+        <v>162</v>
       </c>
       <c r="D12" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E12" s="2" t="s">
-        <v>152</v>
-      </c>
-      <c r="F12" s="2" t="n">
+        <v>163</v>
+      </c>
+      <c r="F12" s="2" t="s">
+        <v>164</v>
+      </c>
+      <c r="G12" s="2" t="n">
         <v>2026</v>
       </c>
-      <c r="G12" s="2" t="n">
+      <c r="H12" s="2" t="n">
         <v>45937</v>
       </c>
-      <c r="H12" s="2" t="s">
-        <v>110</v>
-      </c>
       <c r="I12" s="2" t="s">
-        <v>153</v>
+        <v>121</v>
       </c>
       <c r="J12" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2" t="s">
-        <v>29</v>
-      </c>
+        <v>165</v>
+      </c>
+      <c r="K12" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="L12" s="2"/>
       <c r="M12" s="2" t="s">
-        <v>154</v>
-      </c>
-      <c r="N12" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>166</v>
+      </c>
       <c r="O12" s="2"/>
-      <c r="P12" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="P12" s="2"/>
       <c r="Q12" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="R12" s="2" t="n">
         <v>0</v>
@@ -2552,54 +2671,57 @@
       <c r="S12" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T12" s="2" t="s">
-        <v>73</v>
+      <c r="T12" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="U12" s="2" t="s">
-        <v>33</v>
+        <v>79</v>
+      </c>
+      <c r="V12" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="s">
-        <v>155</v>
+        <v>167</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>156</v>
+        <v>168</v>
       </c>
       <c r="C13" s="2"/>
       <c r="D13" s="2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="E13" s="2" t="s">
-        <v>98</v>
-      </c>
-      <c r="F13" s="2" t="n">
+        <v>107</v>
+      </c>
+      <c r="F13" s="2" t="s">
+        <v>108</v>
+      </c>
+      <c r="G13" s="2" t="n">
         <v>2024</v>
       </c>
-      <c r="G13" s="2" t="n">
+      <c r="H13" s="2" t="n">
         <v>45250</v>
       </c>
-      <c r="H13" s="2" t="s">
-        <v>117</v>
-      </c>
       <c r="I13" s="2" t="s">
-        <v>157</v>
+        <v>128</v>
       </c>
       <c r="J13" s="2" t="s">
-        <v>112</v>
-      </c>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2" t="s">
-        <v>29</v>
-      </c>
+        <v>169</v>
+      </c>
+      <c r="K13" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="L13" s="2"/>
       <c r="M13" s="2" t="s">
-        <v>95</v>
-      </c>
-      <c r="N13" s="2"/>
+        <v>31</v>
+      </c>
+      <c r="N13" s="2" t="s">
+        <v>104</v>
+      </c>
       <c r="O13" s="2"/>
-      <c r="P13" s="2" t="n">
-        <v>0</v>
-      </c>
+      <c r="P13" s="2"/>
       <c r="Q13" s="2" t="n">
         <v>0</v>
       </c>
@@ -2609,11 +2731,14 @@
       <c r="S13" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="T13" s="2" t="s">
-        <v>32</v>
+      <c r="T13" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="U13" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
+      </c>
+      <c r="V13" s="2" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>

</xml_diff>